<commit_message>
Fixed names of total synapse number distributions in SEED and build_network files.
</commit_message>
<xml_diff>
--- a/base_props/V1model_seed_file.xlsx
+++ b/base_props/V1model_seed_file.xlsx
@@ -355,7 +355,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q42"/>
-  <sheetFormatPr defaultColWidth="10.50390625" defaultRowHeight="16" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.51171875" defaultRowHeight="16" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.83"/>
@@ -1805,7 +1805,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="10.50390625" defaultRowHeight="16" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.51171875" defaultRowHeight="16" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="19.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20.66"/>

</xml_diff>

<commit_message>
Switching to radius based construction
</commit_message>
<xml_diff>
--- a/base_props/V1model_seed_file.xlsx
+++ b/base_props/V1model_seed_file.xlsx
@@ -1,20 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shinya.ito/projects/Modeling/biorealistic-v1-model/base_props/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A3BAE00-6983-8049-A969-6C4ED811C985}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE3C331A-08D7-4646-9BB9-81FD21E36611}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="22480" windowHeight="17440" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8140" yWindow="12140" windowWidth="29520" windowHeight="22400" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cell_models" sheetId="1" r:id="rId1"/>
-    <sheet name="general_parameters" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029" refMode="R1C1"/>
   <extLst>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="78">
   <si>
     <t>pop_id</t>
   </si>
@@ -69,9 +68,6 @@
     <t>Relative fraction within ei</t>
   </si>
   <si>
-    <t>base core cell number</t>
-  </si>
-  <si>
     <t>inhibitory fraction</t>
   </si>
   <si>
@@ -258,24 +254,31 @@
     <t>L6</t>
   </si>
   <si>
-    <t>properties</t>
-  </si>
-  <si>
-    <t>values</t>
-  </si>
-  <si>
-    <t>radius</t>
-  </si>
-  <si>
-    <t>core_radius</t>
+    <t>Cells found in EM</t>
+  </si>
+  <si>
+    <t>Density (#/mm^3)</t>
+  </si>
+  <si>
+    <t>Areal density (#/mm^2)</t>
+  </si>
+  <si>
+    <t>Areal Density (#/mm^2)</t>
+  </si>
+  <si>
+    <t>Layer areal density</t>
+  </si>
+  <si>
+    <t>Total</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -306,9 +309,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -643,28 +652,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q42"/>
+  <dimension ref="A1:R48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.33203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="9.1640625" customWidth="1"/>
-    <col min="4" max="4" width="5.1640625" customWidth="1"/>
-    <col min="5" max="5" width="19" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.5" customWidth="1"/>
     <col min="6" max="7" width="14.6640625" customWidth="1"/>
     <col min="8" max="8" width="12.33203125" customWidth="1"/>
-    <col min="9" max="9" width="13" customWidth="1"/>
-    <col min="10" max="10" width="23.1640625" customWidth="1"/>
-    <col min="11" max="11" width="19.83203125" customWidth="1"/>
+    <col min="9" max="9" width="13.5" customWidth="1"/>
+    <col min="10" max="10" width="17.1640625" customWidth="1"/>
+    <col min="11" max="11" width="16.33203125" customWidth="1"/>
     <col min="12" max="12" width="19.33203125" customWidth="1"/>
-    <col min="13" max="13" width="14.83203125" customWidth="1"/>
-    <col min="14" max="14" width="19.1640625" customWidth="1"/>
-    <col min="15" max="15" width="19.5" customWidth="1"/>
-    <col min="16" max="16" width="12.33203125" customWidth="1"/>
-    <col min="17" max="17" width="13.1640625" customWidth="1"/>
+    <col min="13" max="13" width="16.6640625" customWidth="1"/>
+    <col min="14" max="14" width="21.5" customWidth="1"/>
+    <col min="15" max="15" width="19.1640625" customWidth="1"/>
+    <col min="16" max="16" width="19.5" customWidth="1"/>
+    <col min="17" max="17" width="12.33203125" customWidth="1"/>
+    <col min="18" max="18" width="13.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -693,49 +703,52 @@
         <v>8</v>
       </c>
       <c r="J1" t="s">
-        <v>9</v>
+        <v>76</v>
       </c>
       <c r="K1" t="s">
         <v>10</v>
       </c>
       <c r="L1" t="s">
+        <v>9</v>
+      </c>
+      <c r="M1" t="s">
+        <v>74</v>
+      </c>
+      <c r="N1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="O1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="P1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="Q1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="R1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>0</v>
       </c>
       <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
         <v>17</v>
-      </c>
-      <c r="C2" t="s">
-        <v>18</v>
       </c>
       <c r="D2" t="str">
         <f t="shared" ref="D2:D23" si="0">LEFT(B2, 1)</f>
         <v>i</v>
       </c>
       <c r="E2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" t="s">
         <v>19</v>
-      </c>
-      <c r="F2" t="s">
-        <v>20</v>
       </c>
       <c r="H2">
         <f>$C$37</f>
@@ -745,53 +758,58 @@
         <f>$C$38</f>
         <v>169</v>
       </c>
-      <c r="J2">
+      <c r="J2" s="5">
+        <f>$F$38</f>
+        <v>1200</v>
+      </c>
+      <c r="K2">
         <v>1</v>
-      </c>
-      <c r="K2">
-        <v>603</v>
       </c>
       <c r="L2">
         <v>1</v>
       </c>
-      <c r="M2">
-        <f t="shared" ref="M2:M23" si="1">ROUND(K2*J2*IF(EXACT(D2,"i"), L2, 1-L2), 0)</f>
+      <c r="M2" s="4">
+        <f>J2*L2*IF(EXACT(D2,"i"), K2, 1-K2)</f>
+        <v>1200</v>
+      </c>
+      <c r="N2" s="5">
+        <f>ROUND(M2*$B$48, 0)</f>
         <v>603</v>
       </c>
-      <c r="N2">
-        <f t="shared" ref="N2:N23" si="2">ROUND(M2/$J$38*$K$38, 0)</f>
-        <v>2088</v>
-      </c>
       <c r="O2">
-        <f t="shared" ref="O2:O23" si="3">SUM(M2:N2)</f>
-        <v>2691</v>
-      </c>
-      <c r="P2">
+        <f>ROUND(M2*$C$48, 0)</f>
+        <v>1244</v>
+      </c>
+      <c r="P2" s="5">
+        <f>SUM(N2:O2)</f>
+        <v>1847</v>
+      </c>
+      <c r="Q2">
         <v>0.85599999999999998</v>
       </c>
-      <c r="Q2">
+      <c r="R2">
         <v>2808.6819999999998</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s">
         <v>21</v>
-      </c>
-      <c r="C3" t="s">
-        <v>22</v>
       </c>
       <c r="D3" t="str">
         <f t="shared" si="0"/>
         <v>e</v>
       </c>
       <c r="E3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H3">
         <f>$C$38</f>
@@ -801,53 +819,58 @@
         <f>$C$39</f>
         <v>357</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="5">
+        <f>$F$39</f>
+        <v>37099.999999999993</v>
+      </c>
+      <c r="K3">
+        <v>0.1</v>
+      </c>
+      <c r="L3">
         <v>1</v>
       </c>
-      <c r="K3">
-        <v>18648</v>
-      </c>
-      <c r="L3">
-        <v>0.1</v>
-      </c>
-      <c r="M3">
-        <f t="shared" si="1"/>
-        <v>16783</v>
-      </c>
-      <c r="N3">
-        <f t="shared" si="2"/>
-        <v>58114</v>
+      <c r="M3" s="4">
+        <f t="shared" ref="M3:M23" si="1">J3*L3*IF(EXACT(D3,"i"), K3, 1-K3)</f>
+        <v>33389.999999999993</v>
+      </c>
+      <c r="N3" s="5">
+        <f t="shared" ref="N3:N23" si="2">ROUND(M3*$B$48, 0)</f>
+        <v>16784</v>
       </c>
       <c r="O3">
-        <f t="shared" si="3"/>
-        <v>74897</v>
-      </c>
-      <c r="P3">
+        <f t="shared" ref="O3:O23" si="3">ROUND(M3*$C$48, 0)</f>
+        <v>34616</v>
+      </c>
+      <c r="P3" s="5">
+        <f t="shared" ref="P3:P23" si="4">SUM(N3:O3)</f>
+        <v>51400</v>
+      </c>
+      <c r="Q3">
         <v>0.36299999999999999</v>
       </c>
-      <c r="Q3">
+      <c r="R3">
         <v>3815.6819999999998</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D4" t="str">
         <f t="shared" si="0"/>
         <v>i</v>
       </c>
       <c r="E4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H4">
         <f>$C$38</f>
@@ -857,54 +880,59 @@
         <f>$C$39</f>
         <v>357</v>
       </c>
-      <c r="J4">
+      <c r="J4" s="5">
+        <f t="shared" ref="J4:J6" si="5">$F$39</f>
+        <v>37099.999999999993</v>
+      </c>
+      <c r="K4">
+        <v>0.1</v>
+      </c>
+      <c r="L4">
         <f>48/98</f>
         <v>0.48979591836734693</v>
       </c>
-      <c r="K4">
-        <v>18648</v>
-      </c>
-      <c r="L4">
-        <v>0.1</v>
-      </c>
-      <c r="M4">
+      <c r="M4" s="4">
         <f t="shared" si="1"/>
+        <v>1817.1428571428569</v>
+      </c>
+      <c r="N4" s="5">
+        <f t="shared" si="2"/>
         <v>913</v>
-      </c>
-      <c r="N4">
-        <f t="shared" si="2"/>
-        <v>3161</v>
       </c>
       <c r="O4">
         <f t="shared" si="3"/>
-        <v>4074</v>
-      </c>
-      <c r="P4">
+        <v>1884</v>
+      </c>
+      <c r="P4" s="5">
+        <f t="shared" si="4"/>
+        <v>2797</v>
+      </c>
+      <c r="Q4">
         <v>0.53700000000000003</v>
       </c>
-      <c r="Q4">
+      <c r="R4">
         <v>2355.279</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D5" t="str">
         <f t="shared" si="0"/>
         <v>i</v>
       </c>
       <c r="E5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H5">
         <f>$C$38</f>
@@ -914,54 +942,59 @@
         <f>$C$39</f>
         <v>357</v>
       </c>
-      <c r="J5">
+      <c r="J5" s="5">
+        <f t="shared" si="5"/>
+        <v>37099.999999999993</v>
+      </c>
+      <c r="K5">
+        <v>0.1</v>
+      </c>
+      <c r="L5">
         <f>29/98</f>
         <v>0.29591836734693877</v>
       </c>
-      <c r="K5">
-        <v>18648</v>
-      </c>
-      <c r="L5">
-        <v>0.1</v>
-      </c>
-      <c r="M5">
+      <c r="M5" s="4">
         <f t="shared" si="1"/>
+        <v>1097.8571428571427</v>
+      </c>
+      <c r="N5" s="5">
+        <f t="shared" si="2"/>
         <v>552</v>
-      </c>
-      <c r="N5">
-        <f t="shared" si="2"/>
-        <v>1911</v>
       </c>
       <c r="O5">
         <f t="shared" si="3"/>
-        <v>2463</v>
-      </c>
-      <c r="P5">
+        <v>1138</v>
+      </c>
+      <c r="P5" s="5">
+        <f t="shared" si="4"/>
+        <v>1690</v>
+      </c>
+      <c r="Q5">
         <v>0.433</v>
       </c>
-      <c r="Q5">
+      <c r="R5">
         <v>7432.5870000000004</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D6" t="str">
         <f t="shared" si="0"/>
         <v>i</v>
       </c>
       <c r="E6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H6">
         <f>$C$38</f>
@@ -971,447 +1004,487 @@
         <f>$C$39</f>
         <v>357</v>
       </c>
-      <c r="J6">
+      <c r="J6" s="5">
+        <f t="shared" si="5"/>
+        <v>37099.999999999993</v>
+      </c>
+      <c r="K6">
+        <v>0.1</v>
+      </c>
+      <c r="L6">
         <f>21/98</f>
         <v>0.21428571428571427</v>
       </c>
-      <c r="K6">
-        <v>18648</v>
-      </c>
-      <c r="L6">
-        <v>0.1</v>
-      </c>
-      <c r="M6">
+      <c r="M6" s="4">
         <f t="shared" si="1"/>
+        <v>794.99999999999989</v>
+      </c>
+      <c r="N6" s="5">
+        <f t="shared" si="2"/>
         <v>400</v>
-      </c>
-      <c r="N6">
-        <f t="shared" si="2"/>
-        <v>1385</v>
       </c>
       <c r="O6">
         <f t="shared" si="3"/>
-        <v>1785</v>
-      </c>
-      <c r="P6">
+        <v>824</v>
+      </c>
+      <c r="P6" s="5">
+        <f t="shared" si="4"/>
+        <v>1224</v>
+      </c>
+      <c r="Q6">
         <v>0.55000000000000004</v>
       </c>
-      <c r="Q6">
+      <c r="R6">
         <v>5305.1509999999998</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>5</v>
       </c>
       <c r="B7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" t="s">
         <v>30</v>
-      </c>
-      <c r="C7" t="s">
-        <v>31</v>
       </c>
       <c r="D7" t="str">
         <f t="shared" si="0"/>
         <v>e</v>
       </c>
       <c r="E7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H7">
-        <f t="shared" ref="H7:H13" si="4">$C$39</f>
+        <f t="shared" ref="H7:H13" si="6">$C$39</f>
         <v>357</v>
       </c>
       <c r="I7">
-        <f t="shared" ref="I7:I13" si="5">$C$40</f>
+        <f>$C$40</f>
         <v>505</v>
       </c>
-      <c r="J7">
+      <c r="J7" s="5">
+        <f>$F$40</f>
+        <v>38899.999999999993</v>
+      </c>
+      <c r="K7">
+        <v>0.11</v>
+      </c>
+      <c r="L7">
         <v>0.12</v>
       </c>
-      <c r="K7">
-        <v>19553</v>
-      </c>
-      <c r="L7">
-        <v>0.11</v>
-      </c>
-      <c r="M7">
+      <c r="M7" s="4">
         <f t="shared" si="1"/>
+        <v>4154.5199999999995</v>
+      </c>
+      <c r="N7" s="5">
+        <f t="shared" si="2"/>
         <v>2088</v>
-      </c>
-      <c r="N7">
-        <f t="shared" si="2"/>
-        <v>7230</v>
       </c>
       <c r="O7">
         <f t="shared" si="3"/>
-        <v>9318</v>
-      </c>
-      <c r="P7">
+        <v>4307</v>
+      </c>
+      <c r="P7" s="5">
+        <f t="shared" si="4"/>
+        <v>6395</v>
+      </c>
+      <c r="Q7">
         <v>0.34499999999999997</v>
       </c>
-      <c r="Q7">
+      <c r="R7">
         <v>2188.7649999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D8" t="str">
         <f t="shared" si="0"/>
         <v>e</v>
       </c>
       <c r="E8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H8">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>357</v>
       </c>
       <c r="I8">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="I8:I13" si="7">$C$40</f>
         <v>505</v>
       </c>
-      <c r="J8">
+      <c r="J8" s="5">
+        <f t="shared" ref="J8:J13" si="8">$F$40</f>
+        <v>38899.999999999993</v>
+      </c>
+      <c r="K8">
+        <v>0.11</v>
+      </c>
+      <c r="L8">
         <v>0.26</v>
       </c>
-      <c r="K8">
-        <v>19553</v>
-      </c>
-      <c r="L8">
-        <v>0.11</v>
-      </c>
-      <c r="M8">
+      <c r="M8" s="4">
         <f t="shared" si="1"/>
+        <v>9001.4599999999991</v>
+      </c>
+      <c r="N8" s="5">
+        <f t="shared" si="2"/>
         <v>4525</v>
-      </c>
-      <c r="N8">
-        <f t="shared" si="2"/>
-        <v>15669</v>
       </c>
       <c r="O8">
         <f t="shared" si="3"/>
-        <v>20194</v>
-      </c>
-      <c r="P8">
+        <v>9332</v>
+      </c>
+      <c r="P8" s="5">
+        <f t="shared" si="4"/>
+        <v>13857</v>
+      </c>
+      <c r="Q8">
         <v>0.34499999999999997</v>
       </c>
-      <c r="Q8">
+      <c r="R8">
         <v>2188.7649999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D9" t="str">
         <f t="shared" si="0"/>
         <v>e</v>
       </c>
       <c r="E9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H9">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>357</v>
       </c>
       <c r="I9">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>505</v>
       </c>
-      <c r="J9">
+      <c r="J9" s="5">
+        <f t="shared" si="8"/>
+        <v>38899.999999999993</v>
+      </c>
+      <c r="K9">
+        <v>0.11</v>
+      </c>
+      <c r="L9">
         <v>0.3</v>
       </c>
-      <c r="K9">
-        <v>19553</v>
-      </c>
-      <c r="L9">
-        <v>0.11</v>
-      </c>
-      <c r="M9">
+      <c r="M9" s="4">
         <f t="shared" si="1"/>
+        <v>10386.299999999999</v>
+      </c>
+      <c r="N9" s="5">
+        <f t="shared" si="2"/>
         <v>5221</v>
-      </c>
-      <c r="N9">
-        <f t="shared" si="2"/>
-        <v>18079</v>
       </c>
       <c r="O9">
         <f t="shared" si="3"/>
-        <v>23300</v>
-      </c>
-      <c r="P9">
+        <v>10768</v>
+      </c>
+      <c r="P9" s="5">
+        <f t="shared" si="4"/>
+        <v>15989</v>
+      </c>
+      <c r="Q9">
         <v>0.34499999999999997</v>
       </c>
-      <c r="Q9">
+      <c r="R9">
         <v>2188.7649999999999</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D10" t="str">
         <f t="shared" si="0"/>
         <v>e</v>
       </c>
       <c r="E10" t="s">
+        <v>37</v>
+      </c>
+      <c r="F10" t="s">
         <v>38</v>
       </c>
-      <c r="F10" t="s">
-        <v>39</v>
-      </c>
       <c r="H10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>357</v>
       </c>
       <c r="I10">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>505</v>
       </c>
-      <c r="J10">
-        <f>1-SUM($J7:$J9)</f>
+      <c r="J10" s="5">
+        <f t="shared" si="8"/>
+        <v>38899.999999999993</v>
+      </c>
+      <c r="K10">
+        <v>0.11</v>
+      </c>
+      <c r="L10">
+        <f>1-SUM($L7:$L9)</f>
         <v>0.32000000000000006</v>
       </c>
-      <c r="K10">
-        <v>19553</v>
-      </c>
-      <c r="L10">
-        <v>0.11</v>
-      </c>
-      <c r="M10">
+      <c r="M10" s="4">
         <f t="shared" si="1"/>
+        <v>11078.72</v>
+      </c>
+      <c r="N10" s="5">
+        <f t="shared" si="2"/>
         <v>5569</v>
-      </c>
-      <c r="N10">
-        <f t="shared" si="2"/>
-        <v>19284</v>
       </c>
       <c r="O10">
         <f t="shared" si="3"/>
-        <v>24853</v>
-      </c>
-      <c r="P10">
+        <v>11486</v>
+      </c>
+      <c r="P10" s="5">
+        <f t="shared" si="4"/>
+        <v>17055</v>
+      </c>
+      <c r="Q10">
         <v>0.34499999999999997</v>
       </c>
-      <c r="Q10">
+      <c r="R10">
         <v>2188.7649999999999</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D11" t="str">
         <f t="shared" si="0"/>
         <v>i</v>
       </c>
       <c r="E11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H11">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>357</v>
       </c>
       <c r="I11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>505</v>
       </c>
-      <c r="J11">
+      <c r="J11" s="5">
+        <f t="shared" si="8"/>
+        <v>38899.999999999993</v>
+      </c>
+      <c r="K11">
+        <v>0.11</v>
+      </c>
+      <c r="L11">
         <f>16/105</f>
         <v>0.15238095238095239</v>
       </c>
-      <c r="K11">
-        <v>19553</v>
-      </c>
-      <c r="L11">
-        <v>0.11</v>
-      </c>
-      <c r="M11">
+      <c r="M11" s="4">
         <f t="shared" si="1"/>
+        <v>652.03809523809514</v>
+      </c>
+      <c r="N11" s="5">
+        <f t="shared" si="2"/>
         <v>328</v>
-      </c>
-      <c r="N11">
-        <f t="shared" si="2"/>
-        <v>1136</v>
       </c>
       <c r="O11">
         <f t="shared" si="3"/>
-        <v>1464</v>
-      </c>
-      <c r="P11">
+        <v>676</v>
+      </c>
+      <c r="P11" s="5">
+        <f t="shared" si="4"/>
+        <v>1004</v>
+      </c>
+      <c r="Q11">
         <v>0.53700000000000003</v>
       </c>
-      <c r="Q11">
+      <c r="R11">
         <v>2355.279</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D12" t="str">
         <f t="shared" si="0"/>
         <v>i</v>
       </c>
       <c r="E12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H12">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>357</v>
       </c>
       <c r="I12">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>505</v>
       </c>
-      <c r="J12">
+      <c r="J12" s="5">
+        <f t="shared" si="8"/>
+        <v>38899.999999999993</v>
+      </c>
+      <c r="K12">
+        <v>0.11</v>
+      </c>
+      <c r="L12">
         <f>58/105</f>
         <v>0.55238095238095242</v>
       </c>
-      <c r="K12">
-        <v>19553</v>
-      </c>
-      <c r="L12">
-        <v>0.11</v>
-      </c>
-      <c r="M12">
+      <c r="M12" s="4">
         <f t="shared" si="1"/>
+        <v>2363.638095238095</v>
+      </c>
+      <c r="N12" s="5">
+        <f t="shared" si="2"/>
         <v>1188</v>
-      </c>
-      <c r="N12">
-        <f t="shared" si="2"/>
-        <v>4114</v>
       </c>
       <c r="O12">
         <f t="shared" si="3"/>
-        <v>5302</v>
-      </c>
-      <c r="P12">
+        <v>2450</v>
+      </c>
+      <c r="P12" s="5">
+        <f t="shared" si="4"/>
+        <v>3638</v>
+      </c>
+      <c r="Q12">
         <v>0.433</v>
       </c>
-      <c r="Q12">
+      <c r="R12">
         <v>7432.5870000000004</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D13" t="str">
         <f t="shared" si="0"/>
         <v>i</v>
       </c>
       <c r="E13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H13">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>357</v>
       </c>
       <c r="I13">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>505</v>
       </c>
-      <c r="J13">
+      <c r="J13" s="5">
+        <f t="shared" si="8"/>
+        <v>38899.999999999993</v>
+      </c>
+      <c r="K13">
+        <v>0.11</v>
+      </c>
+      <c r="L13">
         <f>31/105</f>
         <v>0.29523809523809524</v>
       </c>
-      <c r="K13">
-        <v>19553</v>
-      </c>
-      <c r="L13">
-        <v>0.11</v>
-      </c>
-      <c r="M13">
+      <c r="M13" s="4">
         <f t="shared" si="1"/>
+        <v>1263.3238095238094</v>
+      </c>
+      <c r="N13" s="5">
+        <f t="shared" si="2"/>
         <v>635</v>
-      </c>
-      <c r="N13">
-        <f t="shared" si="2"/>
-        <v>2199</v>
       </c>
       <c r="O13">
         <f t="shared" si="3"/>
-        <v>2834</v>
-      </c>
-      <c r="P13">
+        <v>1310</v>
+      </c>
+      <c r="P13" s="5">
+        <f t="shared" si="4"/>
+        <v>1945</v>
+      </c>
+      <c r="Q13">
         <v>0.55000000000000004</v>
       </c>
-      <c r="Q13">
+      <c r="R13">
         <v>5305.1509999999998</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>12</v>
       </c>
       <c r="B14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" t="s">
         <v>43</v>
-      </c>
-      <c r="C14" t="s">
-        <v>44</v>
       </c>
       <c r="D14" t="str">
         <f t="shared" si="0"/>
         <v>e</v>
       </c>
       <c r="G14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H14">
         <f>$C$40</f>
@@ -1421,50 +1494,55 @@
         <f>$C$41</f>
         <v>665</v>
       </c>
-      <c r="J14">
+      <c r="J14" s="5">
+        <f>$F$41</f>
+        <v>23000</v>
+      </c>
+      <c r="K14">
+        <v>0.19</v>
+      </c>
+      <c r="L14">
         <v>0.7</v>
       </c>
-      <c r="K14">
-        <v>11561</v>
-      </c>
-      <c r="L14">
-        <v>0.19</v>
-      </c>
-      <c r="M14">
+      <c r="M14" s="4">
         <f t="shared" si="1"/>
+        <v>13041</v>
+      </c>
+      <c r="N14" s="5">
+        <f t="shared" si="2"/>
         <v>6555</v>
-      </c>
-      <c r="N14">
-        <f t="shared" si="2"/>
-        <v>22698</v>
       </c>
       <c r="O14">
         <f t="shared" si="3"/>
-        <v>29253</v>
-      </c>
-      <c r="P14">
+        <v>13520</v>
+      </c>
+      <c r="P14" s="5">
+        <f t="shared" si="4"/>
+        <v>20075</v>
+      </c>
+      <c r="Q14">
         <v>0.33100000000000002</v>
       </c>
-      <c r="Q14">
+      <c r="R14">
         <v>2552.0720000000001</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D15" t="str">
         <f t="shared" si="0"/>
         <v>e</v>
       </c>
       <c r="G15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H15">
         <f>$C$40</f>
@@ -1474,50 +1552,55 @@
         <f>$C$41</f>
         <v>665</v>
       </c>
-      <c r="J15">
+      <c r="J15" s="5">
+        <f t="shared" ref="J15:J19" si="9">$F$41</f>
+        <v>23000</v>
+      </c>
+      <c r="K15">
+        <v>0.19</v>
+      </c>
+      <c r="L15">
         <v>0.26</v>
       </c>
-      <c r="K15">
-        <v>11561</v>
-      </c>
-      <c r="L15">
-        <v>0.19</v>
-      </c>
-      <c r="M15">
+      <c r="M15" s="4">
         <f t="shared" si="1"/>
+        <v>4843.8</v>
+      </c>
+      <c r="N15" s="5">
+        <f t="shared" si="2"/>
         <v>2435</v>
-      </c>
-      <c r="N15">
-        <f t="shared" si="2"/>
-        <v>8432</v>
       </c>
       <c r="O15">
         <f t="shared" si="3"/>
-        <v>10867</v>
-      </c>
-      <c r="P15">
+        <v>5022</v>
+      </c>
+      <c r="P15" s="5">
+        <f t="shared" si="4"/>
+        <v>7457</v>
+      </c>
+      <c r="Q15">
         <v>0.42399999999999999</v>
       </c>
-      <c r="Q15">
+      <c r="R15">
         <v>7406.5460000000003</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C16" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D16" t="str">
         <f t="shared" si="0"/>
         <v>e</v>
       </c>
       <c r="G16" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H16">
         <v>505</v>
@@ -1525,53 +1608,58 @@
       <c r="I16">
         <v>665</v>
       </c>
-      <c r="J16">
+      <c r="J16" s="5">
+        <f t="shared" si="9"/>
+        <v>23000</v>
+      </c>
+      <c r="K16">
+        <v>0.19</v>
+      </c>
+      <c r="L16">
         <v>0.04</v>
       </c>
-      <c r="K16">
-        <v>11561</v>
-      </c>
-      <c r="L16">
-        <v>0.19</v>
-      </c>
-      <c r="M16">
+      <c r="M16" s="4">
         <f t="shared" si="1"/>
+        <v>745.2</v>
+      </c>
+      <c r="N16" s="5">
+        <f t="shared" si="2"/>
         <v>375</v>
-      </c>
-      <c r="N16">
-        <f t="shared" si="2"/>
-        <v>1298</v>
       </c>
       <c r="O16">
         <f t="shared" si="3"/>
-        <v>1673</v>
-      </c>
-      <c r="P16">
+        <v>773</v>
+      </c>
+      <c r="P16" s="5">
+        <f t="shared" si="4"/>
+        <v>1148</v>
+      </c>
+      <c r="Q16">
         <v>1.3759999999999999</v>
       </c>
-      <c r="Q16">
+      <c r="R16">
         <v>679.745</v>
       </c>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>14</v>
       </c>
       <c r="B17" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D17" t="str">
         <f t="shared" si="0"/>
         <v>i</v>
       </c>
       <c r="E17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H17">
         <f>$C$40</f>
@@ -1581,54 +1669,59 @@
         <f>$C$41</f>
         <v>665</v>
       </c>
-      <c r="J17">
+      <c r="J17" s="5">
+        <f t="shared" si="9"/>
+        <v>23000</v>
+      </c>
+      <c r="K17">
+        <v>0.19</v>
+      </c>
+      <c r="L17">
         <f>9/105</f>
         <v>8.5714285714285715E-2</v>
       </c>
-      <c r="K17">
-        <v>11561</v>
-      </c>
-      <c r="L17">
-        <v>0.19</v>
-      </c>
-      <c r="M17">
+      <c r="M17" s="4">
         <f t="shared" si="1"/>
+        <v>374.57142857142861</v>
+      </c>
+      <c r="N17" s="5">
+        <f t="shared" si="2"/>
         <v>188</v>
-      </c>
-      <c r="N17">
-        <f t="shared" si="2"/>
-        <v>651</v>
       </c>
       <c r="O17">
         <f t="shared" si="3"/>
-        <v>839</v>
-      </c>
-      <c r="P17">
+        <v>388</v>
+      </c>
+      <c r="P17" s="5">
+        <f t="shared" si="4"/>
+        <v>576</v>
+      </c>
+      <c r="Q17">
         <v>0.53700000000000003</v>
       </c>
-      <c r="Q17">
+      <c r="R17">
         <v>2355.279</v>
       </c>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>15</v>
       </c>
       <c r="B18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C18" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D18" t="str">
         <f t="shared" si="0"/>
         <v>i</v>
       </c>
       <c r="E18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H18">
         <f>$C$40</f>
@@ -1638,54 +1731,59 @@
         <f>$C$41</f>
         <v>665</v>
       </c>
-      <c r="J18">
+      <c r="J18" s="5">
+        <f t="shared" si="9"/>
+        <v>23000</v>
+      </c>
+      <c r="K18">
+        <v>0.19</v>
+      </c>
+      <c r="L18">
         <f>51/105</f>
         <v>0.48571428571428571</v>
       </c>
-      <c r="K18">
-        <v>11561</v>
-      </c>
-      <c r="L18">
-        <v>0.19</v>
-      </c>
-      <c r="M18">
+      <c r="M18" s="4">
         <f t="shared" si="1"/>
+        <v>2122.5714285714284</v>
+      </c>
+      <c r="N18" s="5">
+        <f t="shared" si="2"/>
         <v>1067</v>
-      </c>
-      <c r="N18">
-        <f t="shared" si="2"/>
-        <v>3695</v>
       </c>
       <c r="O18">
         <f t="shared" si="3"/>
-        <v>4762</v>
-      </c>
-      <c r="P18">
+        <v>2201</v>
+      </c>
+      <c r="P18" s="5">
+        <f t="shared" si="4"/>
+        <v>3268</v>
+      </c>
+      <c r="Q18">
         <v>0.433</v>
       </c>
-      <c r="Q18">
+      <c r="R18">
         <v>7432.5870000000004</v>
       </c>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>16</v>
       </c>
       <c r="B19" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C19" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D19" t="str">
         <f t="shared" si="0"/>
         <v>i</v>
       </c>
       <c r="E19" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H19">
         <f>$C$40</f>
@@ -1695,54 +1793,59 @@
         <f>$C$41</f>
         <v>665</v>
       </c>
-      <c r="J19">
+      <c r="J19" s="5">
+        <f t="shared" si="9"/>
+        <v>23000</v>
+      </c>
+      <c r="K19">
+        <v>0.19</v>
+      </c>
+      <c r="L19">
         <f>45/105</f>
         <v>0.42857142857142855</v>
       </c>
-      <c r="K19">
-        <v>11561</v>
-      </c>
-      <c r="L19">
-        <v>0.19</v>
-      </c>
-      <c r="M19">
+      <c r="M19" s="4">
         <f t="shared" si="1"/>
+        <v>1872.8571428571429</v>
+      </c>
+      <c r="N19" s="5">
+        <f t="shared" si="2"/>
         <v>941</v>
-      </c>
-      <c r="N19">
-        <f t="shared" si="2"/>
-        <v>3258</v>
       </c>
       <c r="O19">
         <f t="shared" si="3"/>
-        <v>4199</v>
-      </c>
-      <c r="P19">
+        <v>1942</v>
+      </c>
+      <c r="P19" s="5">
+        <f t="shared" si="4"/>
+        <v>2883</v>
+      </c>
+      <c r="Q19">
         <v>0.55000000000000004</v>
       </c>
-      <c r="Q19">
+      <c r="R19">
         <v>5305.1509999999998</v>
       </c>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>17</v>
       </c>
       <c r="B20" t="s">
+        <v>52</v>
+      </c>
+      <c r="C20" t="s">
         <v>53</v>
-      </c>
-      <c r="C20" t="s">
-        <v>54</v>
       </c>
       <c r="D20" t="str">
         <f t="shared" si="0"/>
         <v>e</v>
       </c>
       <c r="E20" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H20">
         <f>$C$41</f>
@@ -1752,53 +1855,58 @@
         <f>$C$42</f>
         <v>829</v>
       </c>
-      <c r="J20">
+      <c r="J20" s="5">
+        <f>$F$42</f>
+        <v>32200.000000000004</v>
+      </c>
+      <c r="K20">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="L20">
         <v>1</v>
       </c>
-      <c r="K20">
-        <v>16185</v>
-      </c>
-      <c r="L20">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="M20">
+      <c r="M20" s="4">
         <f t="shared" si="1"/>
-        <v>15052</v>
-      </c>
-      <c r="N20">
+        <v>29946</v>
+      </c>
+      <c r="N20" s="5">
         <f t="shared" si="2"/>
-        <v>52120</v>
+        <v>15053</v>
       </c>
       <c r="O20">
         <f t="shared" si="3"/>
-        <v>67172</v>
-      </c>
-      <c r="P20">
+        <v>31046</v>
+      </c>
+      <c r="P20" s="5">
+        <f t="shared" si="4"/>
+        <v>46099</v>
+      </c>
+      <c r="Q20">
         <v>0.24099999999999999</v>
       </c>
-      <c r="Q20">
+      <c r="R20">
         <v>2292.098</v>
       </c>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>18</v>
       </c>
       <c r="B21" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D21" t="str">
         <f t="shared" si="0"/>
         <v>i</v>
       </c>
       <c r="E21" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F21" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H21">
         <f>$C$41</f>
@@ -1808,54 +1916,59 @@
         <f>$C$42</f>
         <v>829</v>
       </c>
-      <c r="J21">
+      <c r="J21" s="5">
+        <f t="shared" ref="J21:J23" si="10">$F$42</f>
+        <v>32200.000000000004</v>
+      </c>
+      <c r="K21">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="L21">
         <f>8/96</f>
         <v>8.3333333333333329E-2</v>
       </c>
-      <c r="K21">
-        <v>16185</v>
-      </c>
-      <c r="L21">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="M21">
+      <c r="M21" s="4">
         <f t="shared" si="1"/>
+        <v>187.83333333333337</v>
+      </c>
+      <c r="N21" s="5">
+        <f t="shared" si="2"/>
         <v>94</v>
-      </c>
-      <c r="N21">
-        <f t="shared" si="2"/>
-        <v>325</v>
       </c>
       <c r="O21">
         <f t="shared" si="3"/>
-        <v>419</v>
-      </c>
-      <c r="P21">
+        <v>195</v>
+      </c>
+      <c r="P21" s="5">
+        <f t="shared" si="4"/>
+        <v>289</v>
+      </c>
+      <c r="Q21">
         <v>0.53700000000000003</v>
       </c>
-      <c r="Q21">
+      <c r="R21">
         <v>2355.279</v>
       </c>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>19</v>
       </c>
       <c r="B22" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C22" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D22" t="str">
         <f t="shared" si="0"/>
         <v>i</v>
       </c>
       <c r="E22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H22">
         <f>$C$41</f>
@@ -1865,54 +1978,59 @@
         <f>$C$42</f>
         <v>829</v>
       </c>
-      <c r="J22">
+      <c r="J22" s="5">
+        <f t="shared" si="10"/>
+        <v>32200.000000000004</v>
+      </c>
+      <c r="K22">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="L22">
         <f>44/96</f>
         <v>0.45833333333333331</v>
       </c>
-      <c r="K22">
-        <v>16185</v>
-      </c>
-      <c r="L22">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="M22">
+      <c r="M22" s="4">
         <f t="shared" si="1"/>
+        <v>1033.0833333333335</v>
+      </c>
+      <c r="N22" s="5">
+        <f t="shared" si="2"/>
         <v>519</v>
-      </c>
-      <c r="N22">
-        <f t="shared" si="2"/>
-        <v>1797</v>
       </c>
       <c r="O22">
         <f t="shared" si="3"/>
-        <v>2316</v>
-      </c>
-      <c r="P22">
+        <v>1071</v>
+      </c>
+      <c r="P22" s="5">
+        <f t="shared" si="4"/>
+        <v>1590</v>
+      </c>
+      <c r="Q22">
         <v>0.433</v>
       </c>
-      <c r="Q22">
+      <c r="R22">
         <v>7432.5870000000004</v>
       </c>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>20</v>
       </c>
       <c r="B23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C23" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D23" t="str">
         <f t="shared" si="0"/>
         <v>i</v>
       </c>
       <c r="E23" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F23" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H23">
         <f>$C$41</f>
@@ -1922,72 +2040,84 @@
         <f>$C$42</f>
         <v>829</v>
       </c>
-      <c r="J23">
+      <c r="J23" s="5">
+        <f t="shared" si="10"/>
+        <v>32200.000000000004</v>
+      </c>
+      <c r="K23">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="L23">
         <f>44/96</f>
         <v>0.45833333333333331</v>
       </c>
-      <c r="K23">
-        <v>16185</v>
-      </c>
-      <c r="L23">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="M23">
+      <c r="M23" s="4">
         <f t="shared" si="1"/>
+        <v>1033.0833333333335</v>
+      </c>
+      <c r="N23" s="5">
+        <f t="shared" si="2"/>
         <v>519</v>
-      </c>
-      <c r="N23">
-        <f t="shared" si="2"/>
-        <v>1797</v>
       </c>
       <c r="O23">
         <f t="shared" si="3"/>
-        <v>2316</v>
-      </c>
-      <c r="P23">
+        <v>1071</v>
+      </c>
+      <c r="P23" s="5">
+        <f t="shared" si="4"/>
+        <v>1590</v>
+      </c>
+      <c r="Q23">
         <v>0.55000000000000004</v>
       </c>
-      <c r="Q23">
+      <c r="R23">
         <v>5305.1509999999998</v>
       </c>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="M25">
-        <f>SUM(M2:M23)</f>
-        <v>66550</v>
-      </c>
-      <c r="N25">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="M24" s="3"/>
+      <c r="N24" s="3"/>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="M25" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="N25" s="5">
         <f>SUM(N2:N23)</f>
-        <v>230441</v>
+        <v>66552</v>
       </c>
       <c r="O25">
         <f>SUM(O2:O23)</f>
-        <v>296991</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+        <v>137264</v>
+      </c>
+      <c r="P25">
+        <f>SUM(P2:P23)</f>
+        <v>203816</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36" t="s">
         <v>59</v>
       </c>
-      <c r="B36" t="s">
+      <c r="C36" t="s">
         <v>60</v>
       </c>
-      <c r="C36" t="s">
-        <v>61</v>
-      </c>
-      <c r="I36" t="s">
-        <v>62</v>
-      </c>
-      <c r="J36" t="s">
-        <v>63</v>
-      </c>
-      <c r="K36" t="s">
+      <c r="D36" t="s">
+        <v>72</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F36" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
         <v>64</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
-        <v>65</v>
       </c>
       <c r="B37">
         <v>50</v>
@@ -1996,19 +2126,10 @@
         <f>SUM($B$37:$B37)</f>
         <v>50</v>
       </c>
-      <c r="I37" t="s">
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
         <v>66</v>
-      </c>
-      <c r="J37">
-        <v>0.4</v>
-      </c>
-      <c r="K37">
-        <v>0.84499999999999997</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
-        <v>67</v>
       </c>
       <c r="B38">
         <v>119</v>
@@ -2017,21 +2138,21 @@
         <f>SUM($B$37:$B38)</f>
         <v>169</v>
       </c>
-      <c r="I38" t="s">
+      <c r="D38">
+        <v>12</v>
+      </c>
+      <c r="E38" s="5">
+        <f>D38/B38 * 1000 * 10 * 10</f>
+        <v>10084.033613445377</v>
+      </c>
+      <c r="F38">
+        <f>E38*B38/1000</f>
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
         <v>68</v>
-      </c>
-      <c r="J38" s="1">
-        <f>J37^2*PI()</f>
-        <v>0.50265482457436694</v>
-      </c>
-      <c r="K38" s="1">
-        <f>K37^2*PI() - J37^2*PI()</f>
-        <v>1.7405208699050847</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A39" t="s">
-        <v>69</v>
       </c>
       <c r="B39">
         <v>188</v>
@@ -2040,10 +2161,21 @@
         <f>SUM($B$37:$B39)</f>
         <v>357</v>
       </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="D39">
+        <v>371</v>
+      </c>
+      <c r="E39" s="5">
+        <f t="shared" ref="E39:E42" si="11">D39/B39 * 1000 * 10 * 10</f>
+        <v>197340.42553191487</v>
+      </c>
+      <c r="F39">
+        <f t="shared" ref="F39:F42" si="12">E39*B39/1000</f>
+        <v>37099.999999999993</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B40">
         <v>148</v>
@@ -2052,10 +2184,21 @@
         <f>SUM($B$37:$B40)</f>
         <v>505</v>
       </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="D40">
+        <v>389</v>
+      </c>
+      <c r="E40" s="5">
+        <f t="shared" si="11"/>
+        <v>262837.83783783781</v>
+      </c>
+      <c r="F40">
+        <f t="shared" si="12"/>
+        <v>38899.999999999993</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B41">
         <v>160</v>
@@ -2064,10 +2207,21 @@
         <f>SUM($B$37:$B41)</f>
         <v>665</v>
       </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="D41">
+        <v>230</v>
+      </c>
+      <c r="E41" s="5">
+        <f t="shared" si="11"/>
+        <v>143750</v>
+      </c>
+      <c r="F41">
+        <f t="shared" si="12"/>
+        <v>23000</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B42">
         <v>164</v>
@@ -2076,44 +2230,51 @@
         <f>SUM($B$37:$B42)</f>
         <v>829</v>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
-  <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="19.33203125" customWidth="1"/>
-    <col min="2" max="2" width="20.6640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>73</v>
-      </c>
-      <c r="B1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B2">
-        <v>845</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>76</v>
-      </c>
-      <c r="B3">
-        <v>400</v>
+      <c r="D42">
+        <v>322</v>
+      </c>
+      <c r="E42" s="5">
+        <f t="shared" si="11"/>
+        <v>196341.46341463417</v>
+      </c>
+      <c r="F42">
+        <f t="shared" si="12"/>
+        <v>32200.000000000004</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>61</v>
+      </c>
+      <c r="B46" t="s">
+        <v>62</v>
+      </c>
+      <c r="C46" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>65</v>
+      </c>
+      <c r="B47">
+        <v>0.4</v>
+      </c>
+      <c r="C47">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>67</v>
+      </c>
+      <c r="B48" s="1">
+        <f>B47^2*PI()</f>
+        <v>0.50265482457436694</v>
+      </c>
+      <c r="C48" s="1">
+        <f>C47^2*PI() - B47^2*PI()</f>
+        <v>1.0367255756846314</v>
       </c>
     </row>
   </sheetData>

</xml_diff>